<commit_message>
enhance close pop up
</commit_message>
<xml_diff>
--- a/test-data/order.xlsx
+++ b/test-data/order.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
   <si>
     <t>scenario</t>
   </si>
@@ -75,20 +75,29 @@
     <t>Pilih Charger</t>
   </si>
   <si>
-    <t>Customer berhasil melakukan order charge EVCS</t>
-  </si>
-  <si>
     <t>voucherCode</t>
   </si>
   <si>
-    <t>EVY7MJ</t>
+    <t>inputKWh</t>
+  </si>
+  <si>
+    <t>ODR002</t>
+  </si>
+  <si>
+    <t>Customer gagal melakukan pemesanan EV Charging karena kode voucher invalid</t>
+  </si>
+  <si>
+    <t>Confirm Payment &amp; Submit Order</t>
+  </si>
+  <si>
+    <t>EVCSKU</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,6 +132,27 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="3">
@@ -167,7 +197,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -201,6 +231,21 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -483,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" style="1" customWidth="1"/>
@@ -492,11 +537,11 @@
     <col min="4" max="4" width="99.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.140625" style="1" customWidth="1"/>
-    <col min="7" max="8" width="16.28515625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.7109375" style="1"/>
+    <col min="7" max="9" width="16.28515625" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="10" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="10" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>8</v>
       </c>
@@ -519,33 +564,40 @@
         <v>9</v>
       </c>
       <c r="H1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="6" t="s">
+    <row r="2" spans="1:9" s="15" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="C2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="G2" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="12"/>
+    </row>
+    <row r="3" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="7"/>
@@ -554,8 +606,9 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
-    </row>
-    <row r="4" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
@@ -564,8 +617,9 @@
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="7"/>
@@ -574,8 +628,9 @@
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="7"/>
@@ -584,8 +639,9 @@
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="7"/>
@@ -594,8 +650,9 @@
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
-    </row>
-    <row r="8" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="7"/>
@@ -604,8 +661,9 @@
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
-    </row>
-    <row r="9" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="7"/>
@@ -614,8 +672,9 @@
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
-    </row>
-    <row r="10" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="7"/>
@@ -624,8 +683,9 @@
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
-    </row>
-    <row r="11" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="7"/>
@@ -634,6 +694,7 @@
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>